<commit_message>
modified:   .DS_Store 	modified:   code/pwmSine.cpp 	modified:   code/spwm.xlsx 	modified:   design-controller.md 	modified:   pic/.DS_Store
</commit_message>
<xml_diff>
--- a/code/spwm.xlsx
+++ b/code/spwm.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/margabudi/Documents/hardware/ESU/code/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79D1F63C-F3F0-2D4E-AF16-47027EE8FF03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FC0EC60-8810-3142-B53B-A14B9B392326}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" activeTab="1" xr2:uid="{E8B53389-6343-9547-92DC-AE53BEF90E60}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" activeTab="1" xr2:uid="{E8B53389-6343-9547-92DC-AE53BEF90E60}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1266,9 +1266,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1281,6 +1278,9 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -8143,72 +8143,72 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="3" t="s">
         <v>356</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="4" t="s">
         <v>357</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="4" t="s">
         <v>358</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="4" t="s">
         <v>359</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F1" s="4" t="s">
         <v>360</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="G1" s="4" t="s">
         <v>361</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="H1" s="4" t="s">
         <v>362</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="I1" s="4" t="s">
         <v>363</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="J1" s="4" t="s">
         <v>364</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="K1" s="4" t="s">
         <v>365</v>
       </c>
-      <c r="L1" s="5" t="s">
+      <c r="L1" s="4" t="s">
         <v>366</v>
       </c>
-      <c r="M1" s="5" t="s">
+      <c r="M1" s="4" t="s">
         <v>367</v>
       </c>
-      <c r="N1" s="5" t="s">
+      <c r="N1" s="4" t="s">
         <v>368</v>
       </c>
-      <c r="O1" s="5" t="s">
+      <c r="O1" s="4" t="s">
         <v>369</v>
       </c>
-      <c r="P1" s="5" t="s">
+      <c r="P1" s="4" t="s">
         <v>370</v>
       </c>
-      <c r="Q1" s="5" t="s">
+      <c r="Q1" s="4" t="s">
         <v>371</v>
       </c>
-      <c r="R1" s="5" t="s">
+      <c r="R1" s="4" t="s">
         <v>372</v>
       </c>
-      <c r="S1" s="5" t="s">
+      <c r="S1" s="4" t="s">
         <v>373</v>
       </c>
-      <c r="T1" s="5" t="s">
+      <c r="T1" s="4" t="s">
         <v>374</v>
       </c>
-      <c r="U1" s="5" t="s">
+      <c r="U1" s="4" t="s">
         <v>375</v>
       </c>
-      <c r="V1" s="5" t="s">
+      <c r="V1" s="4" t="s">
         <v>376</v>
       </c>
     </row>
     <row r="2" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B2" s="3">
+      <c r="B2" s="9">
         <v>2</v>
       </c>
       <c r="C2" s="2">
@@ -8273,7 +8273,7 @@
       </c>
     </row>
     <row r="3" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B3" s="3"/>
+      <c r="B3" s="9"/>
       <c r="C3" s="1">
         <f>C2*255</f>
         <v>128.01</v>
@@ -8356,7 +8356,7 @@
       </c>
     </row>
     <row r="4" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B4" s="3">
+      <c r="B4" s="9">
         <v>10</v>
       </c>
       <c r="C4" s="2">
@@ -8421,7 +8421,7 @@
       </c>
     </row>
     <row r="5" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B5" s="3"/>
+      <c r="B5" s="9"/>
       <c r="C5" s="1">
         <f>C4*255</f>
         <v>129.54</v>
@@ -8504,7 +8504,7 @@
       </c>
     </row>
     <row r="6" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B6" s="3">
+      <c r="B6" s="9">
         <v>25</v>
       </c>
       <c r="C6" s="2">
@@ -8569,7 +8569,7 @@
       </c>
     </row>
     <row r="7" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B7" s="3"/>
+      <c r="B7" s="9"/>
       <c r="C7" s="1">
         <f>C6*255</f>
         <v>132.6</v>
@@ -8652,7 +8652,7 @@
       </c>
     </row>
     <row r="8" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B8" s="3">
+      <c r="B8" s="9">
         <v>50</v>
       </c>
       <c r="C8" s="2">
@@ -8717,7 +8717,7 @@
       </c>
     </row>
     <row r="9" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B9" s="3"/>
+      <c r="B9" s="9"/>
       <c r="C9" s="1">
         <f>C8*255</f>
         <v>138.21</v>
@@ -8800,7 +8800,7 @@
       </c>
     </row>
     <row r="10" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B10" s="3">
+      <c r="B10" s="9">
         <v>100</v>
       </c>
       <c r="C10" s="2">
@@ -8865,7 +8865,7 @@
       </c>
     </row>
     <row r="11" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B11" s="3"/>
+      <c r="B11" s="9"/>
       <c r="C11" s="1">
         <f t="shared" ref="C11:V11" si="40">C10*255</f>
         <v>151.215</v>
@@ -8970,72 +8970,72 @@
       <c r="V12" s="1"/>
     </row>
     <row r="13" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B13" s="6" t="s">
+      <c r="B13" s="5" t="s">
         <v>356</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="C13" s="4" t="s">
         <v>357</v>
       </c>
-      <c r="D13" s="5" t="s">
+      <c r="D13" s="4" t="s">
         <v>358</v>
       </c>
-      <c r="E13" s="5" t="s">
+      <c r="E13" s="4" t="s">
         <v>359</v>
       </c>
-      <c r="F13" s="5" t="s">
+      <c r="F13" s="4" t="s">
         <v>360</v>
       </c>
-      <c r="G13" s="5" t="s">
+      <c r="G13" s="4" t="s">
         <v>361</v>
       </c>
-      <c r="H13" s="5" t="s">
+      <c r="H13" s="4" t="s">
         <v>362</v>
       </c>
-      <c r="I13" s="5" t="s">
+      <c r="I13" s="4" t="s">
         <v>363</v>
       </c>
-      <c r="J13" s="5" t="s">
+      <c r="J13" s="4" t="s">
         <v>364</v>
       </c>
-      <c r="K13" s="5" t="s">
+      <c r="K13" s="4" t="s">
         <v>365</v>
       </c>
-      <c r="L13" s="5" t="s">
+      <c r="L13" s="4" t="s">
         <v>366</v>
       </c>
-      <c r="M13" s="5" t="s">
+      <c r="M13" s="4" t="s">
         <v>367</v>
       </c>
-      <c r="N13" s="5" t="s">
+      <c r="N13" s="4" t="s">
         <v>368</v>
       </c>
-      <c r="O13" s="5" t="s">
+      <c r="O13" s="4" t="s">
         <v>369</v>
       </c>
-      <c r="P13" s="5" t="s">
+      <c r="P13" s="4" t="s">
         <v>370</v>
       </c>
-      <c r="Q13" s="5" t="s">
+      <c r="Q13" s="4" t="s">
         <v>371</v>
       </c>
-      <c r="R13" s="5" t="s">
+      <c r="R13" s="4" t="s">
         <v>372</v>
       </c>
-      <c r="S13" s="5" t="s">
+      <c r="S13" s="4" t="s">
         <v>373</v>
       </c>
-      <c r="T13" s="5" t="s">
+      <c r="T13" s="4" t="s">
         <v>374</v>
       </c>
-      <c r="U13" s="5" t="s">
+      <c r="U13" s="4" t="s">
         <v>375</v>
       </c>
-      <c r="V13" s="5" t="s">
+      <c r="V13" s="4" t="s">
         <v>376</v>
       </c>
     </row>
     <row r="14" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B14" s="7">
+      <c r="B14" s="6">
         <v>1</v>
       </c>
       <c r="C14" s="1">
@@ -9120,92 +9120,92 @@
       </c>
     </row>
     <row r="15" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B15" s="8">
+      <c r="B15" s="7">
         <v>2</v>
       </c>
-      <c r="C15" s="9">
+      <c r="C15" s="8">
         <f t="shared" si="41"/>
         <v>127.9743</v>
       </c>
-      <c r="D15" s="9">
+      <c r="D15" s="8">
         <f t="shared" si="41"/>
         <v>128.84129999999999</v>
       </c>
-      <c r="E15" s="9">
+      <c r="E15" s="8">
         <f t="shared" si="41"/>
         <v>129.5145</v>
       </c>
-      <c r="F15" s="9">
+      <c r="F15" s="8">
         <f t="shared" si="41"/>
         <v>129.91739999999999</v>
       </c>
-      <c r="G15" s="9">
+      <c r="G15" s="8">
         <f t="shared" si="41"/>
         <v>130.05000000000001</v>
       </c>
-      <c r="H15" s="9">
+      <c r="H15" s="8">
         <f t="shared" si="41"/>
         <v>129.93270000000001</v>
       </c>
-      <c r="I15" s="9">
+      <c r="I15" s="8">
         <f t="shared" si="41"/>
         <v>129.60120000000001</v>
       </c>
-      <c r="J15" s="9">
+      <c r="J15" s="8">
         <f t="shared" si="41"/>
         <v>129.11670000000001</v>
       </c>
-      <c r="K15" s="9">
+      <c r="K15" s="8">
         <f t="shared" si="41"/>
         <v>128.51490000000001</v>
       </c>
-      <c r="L15" s="9">
+      <c r="L15" s="8">
         <f t="shared" si="41"/>
         <v>127.8468</v>
       </c>
-      <c r="M15" s="9">
+      <c r="M15" s="8">
         <f t="shared" si="41"/>
         <v>127.1532</v>
       </c>
-      <c r="N15" s="9">
+      <c r="N15" s="8">
         <f t="shared" si="41"/>
         <v>126.4851</v>
       </c>
-      <c r="O15" s="9">
+      <c r="O15" s="8">
         <f t="shared" si="41"/>
         <v>125.88330000000001</v>
       </c>
-      <c r="P15" s="9">
+      <c r="P15" s="8">
         <f t="shared" si="41"/>
         <v>125.39879999999999</v>
       </c>
-      <c r="Q15" s="9">
+      <c r="Q15" s="8">
         <f t="shared" si="41"/>
         <v>125.0673</v>
       </c>
-      <c r="R15" s="9">
+      <c r="R15" s="8">
         <f t="shared" si="41"/>
         <v>124.95</v>
       </c>
-      <c r="S15" s="9">
+      <c r="S15" s="8">
         <f t="shared" si="42"/>
         <v>125.0826</v>
       </c>
-      <c r="T15" s="9">
+      <c r="T15" s="8">
         <f t="shared" si="42"/>
         <v>125.4855</v>
       </c>
-      <c r="U15" s="9">
+      <c r="U15" s="8">
         <f t="shared" si="42"/>
         <v>126.1587</v>
       </c>
-      <c r="V15" s="9">
+      <c r="V15" s="8">
         <f t="shared" si="42"/>
         <v>127.0257</v>
       </c>
     </row>
     <row r="16" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B16" s="7">
+      <c r="B16" s="6">
         <v>3</v>
       </c>
       <c r="C16" s="1">
@@ -9290,7 +9290,7 @@
       </c>
     </row>
     <row r="17" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B17" s="7">
+      <c r="B17" s="6">
         <v>4</v>
       </c>
       <c r="C17" s="1">
@@ -9375,7 +9375,7 @@
       </c>
     </row>
     <row r="18" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B18" s="7">
+      <c r="B18" s="6">
         <v>5</v>
       </c>
       <c r="C18" s="1">
@@ -9460,7 +9460,7 @@
       </c>
     </row>
     <row r="19" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B19" s="7">
+      <c r="B19" s="6">
         <v>6</v>
       </c>
       <c r="C19" s="1">
@@ -9545,7 +9545,7 @@
       </c>
     </row>
     <row r="20" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B20" s="7">
+      <c r="B20" s="6">
         <v>7</v>
       </c>
       <c r="C20" s="1">
@@ -9630,7 +9630,7 @@
       </c>
     </row>
     <row r="21" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B21" s="7">
+      <c r="B21" s="6">
         <v>8</v>
       </c>
       <c r="C21" s="1">
@@ -9715,7 +9715,7 @@
       </c>
     </row>
     <row r="22" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B22" s="7">
+      <c r="B22" s="6">
         <v>9</v>
       </c>
       <c r="C22" s="1">
@@ -9800,92 +9800,92 @@
       </c>
     </row>
     <row r="23" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B23" s="8">
+      <c r="B23" s="7">
         <v>10</v>
       </c>
-      <c r="C23" s="9">
+      <c r="C23" s="8">
         <f t="shared" si="41"/>
         <v>129.8715</v>
       </c>
-      <c r="D23" s="9">
+      <c r="D23" s="8">
         <f t="shared" si="41"/>
         <v>134.20650000000001</v>
       </c>
-      <c r="E23" s="9">
+      <c r="E23" s="8">
         <f t="shared" si="41"/>
         <v>137.57249999999999</v>
       </c>
-      <c r="F23" s="9">
+      <c r="F23" s="8">
         <f t="shared" si="41"/>
         <v>139.58699999999999</v>
       </c>
-      <c r="G23" s="9">
+      <c r="G23" s="8">
         <f t="shared" si="41"/>
         <v>140.25</v>
       </c>
-      <c r="H23" s="9">
+      <c r="H23" s="8">
         <f t="shared" si="41"/>
         <v>139.6635</v>
       </c>
-      <c r="I23" s="9">
+      <c r="I23" s="8">
         <f t="shared" si="41"/>
         <v>138.006</v>
       </c>
-      <c r="J23" s="9">
+      <c r="J23" s="8">
         <f t="shared" si="41"/>
         <v>135.58350000000002</v>
       </c>
-      <c r="K23" s="9">
+      <c r="K23" s="8">
         <f t="shared" si="41"/>
         <v>132.5745</v>
       </c>
-      <c r="L23" s="9">
+      <c r="L23" s="8">
         <f t="shared" si="41"/>
         <v>129.23400000000001</v>
       </c>
-      <c r="M23" s="9">
+      <c r="M23" s="8">
         <f t="shared" si="41"/>
         <v>125.76600000000001</v>
       </c>
-      <c r="N23" s="9">
+      <c r="N23" s="8">
         <f t="shared" si="41"/>
         <v>122.4255</v>
       </c>
-      <c r="O23" s="9">
+      <c r="O23" s="8">
         <f t="shared" si="41"/>
         <v>119.4165</v>
       </c>
-      <c r="P23" s="9">
+      <c r="P23" s="8">
         <f t="shared" si="41"/>
         <v>116.994</v>
       </c>
-      <c r="Q23" s="9">
+      <c r="Q23" s="8">
         <f t="shared" si="41"/>
         <v>115.3365</v>
       </c>
-      <c r="R23" s="9">
+      <c r="R23" s="8">
         <f t="shared" si="41"/>
         <v>114.75</v>
       </c>
-      <c r="S23" s="9">
+      <c r="S23" s="8">
         <f t="shared" si="42"/>
         <v>115.413</v>
       </c>
-      <c r="T23" s="9">
+      <c r="T23" s="8">
         <f t="shared" si="42"/>
         <v>117.42749999999999</v>
       </c>
-      <c r="U23" s="9">
+      <c r="U23" s="8">
         <f t="shared" si="42"/>
         <v>120.79349999999999</v>
       </c>
-      <c r="V23" s="9">
+      <c r="V23" s="8">
         <f t="shared" si="42"/>
         <v>125.1285</v>
       </c>
     </row>
     <row r="24" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B24" s="7">
+      <c r="B24" s="6">
         <v>11</v>
       </c>
       <c r="C24" s="1">
@@ -9970,7 +9970,7 @@
       </c>
     </row>
     <row r="25" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B25" s="7">
+      <c r="B25" s="6">
         <v>12</v>
       </c>
       <c r="C25" s="1">
@@ -10055,7 +10055,7 @@
       </c>
     </row>
     <row r="26" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B26" s="7">
+      <c r="B26" s="6">
         <v>13</v>
       </c>
       <c r="C26" s="1">
@@ -10140,7 +10140,7 @@
       </c>
     </row>
     <row r="27" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B27" s="7">
+      <c r="B27" s="6">
         <v>14</v>
       </c>
       <c r="C27" s="1">
@@ -10225,7 +10225,7 @@
       </c>
     </row>
     <row r="28" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B28" s="7">
+      <c r="B28" s="6">
         <v>15</v>
       </c>
       <c r="C28" s="1">
@@ -10310,7 +10310,7 @@
       </c>
     </row>
     <row r="29" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B29" s="7">
+      <c r="B29" s="6">
         <v>16</v>
       </c>
       <c r="C29" s="1">
@@ -10395,7 +10395,7 @@
       </c>
     </row>
     <row r="30" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B30" s="7">
+      <c r="B30" s="6">
         <v>17</v>
       </c>
       <c r="C30" s="1">
@@ -10480,7 +10480,7 @@
       </c>
     </row>
     <row r="31" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B31" s="7">
+      <c r="B31" s="6">
         <v>18</v>
       </c>
       <c r="C31" s="1">
@@ -10565,7 +10565,7 @@
       </c>
     </row>
     <row r="32" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B32" s="7">
+      <c r="B32" s="6">
         <v>19</v>
       </c>
       <c r="C32" s="1">
@@ -10650,7 +10650,7 @@
       </c>
     </row>
     <row r="33" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B33" s="7">
+      <c r="B33" s="6">
         <v>20</v>
       </c>
       <c r="C33" s="1">
@@ -10735,7 +10735,7 @@
       </c>
     </row>
     <row r="34" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B34" s="7">
+      <c r="B34" s="6">
         <v>21</v>
       </c>
       <c r="C34" s="1">
@@ -10820,7 +10820,7 @@
       </c>
     </row>
     <row r="35" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B35" s="7">
+      <c r="B35" s="6">
         <v>22</v>
       </c>
       <c r="C35" s="1">
@@ -10905,7 +10905,7 @@
       </c>
     </row>
     <row r="36" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B36" s="7">
+      <c r="B36" s="6">
         <v>23</v>
       </c>
       <c r="C36" s="1">
@@ -10990,7 +10990,7 @@
       </c>
     </row>
     <row r="37" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B37" s="7">
+      <c r="B37" s="6">
         <v>24</v>
       </c>
       <c r="C37" s="1">
@@ -11075,92 +11075,92 @@
       </c>
     </row>
     <row r="38" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B38" s="8">
+      <c r="B38" s="7">
         <v>25</v>
       </c>
-      <c r="C38" s="9">
+      <c r="C38" s="8">
         <f t="shared" si="44"/>
         <v>133.42875000000001</v>
       </c>
-      <c r="D38" s="9">
+      <c r="D38" s="8">
         <f t="shared" si="44"/>
         <v>144.26625000000001</v>
       </c>
-      <c r="E38" s="9">
+      <c r="E38" s="8">
         <f t="shared" si="44"/>
         <v>152.68125000000001</v>
       </c>
-      <c r="F38" s="9">
+      <c r="F38" s="8">
         <f t="shared" si="44"/>
         <v>157.7175</v>
       </c>
-      <c r="G38" s="9">
+      <c r="G38" s="8">
         <f t="shared" si="44"/>
         <v>159.375</v>
       </c>
-      <c r="H38" s="9">
+      <c r="H38" s="8">
         <f t="shared" si="44"/>
         <v>157.90875</v>
       </c>
-      <c r="I38" s="9">
+      <c r="I38" s="8">
         <f t="shared" si="44"/>
         <v>153.76499999999999</v>
       </c>
-      <c r="J38" s="9">
+      <c r="J38" s="8">
         <f t="shared" si="44"/>
         <v>147.70875000000001</v>
       </c>
-      <c r="K38" s="9">
+      <c r="K38" s="8">
         <f t="shared" si="44"/>
         <v>140.18625</v>
       </c>
-      <c r="L38" s="9">
+      <c r="L38" s="8">
         <f t="shared" si="44"/>
         <v>131.83499999999998</v>
       </c>
-      <c r="M38" s="9">
+      <c r="M38" s="8">
         <f t="shared" si="44"/>
         <v>123.16500000000001</v>
       </c>
-      <c r="N38" s="9">
+      <c r="N38" s="8">
         <f t="shared" si="44"/>
         <v>114.81375</v>
       </c>
-      <c r="O38" s="9">
+      <c r="O38" s="8">
         <f t="shared" si="44"/>
         <v>107.29125000000001</v>
       </c>
-      <c r="P38" s="9">
+      <c r="P38" s="8">
         <f t="shared" si="44"/>
         <v>101.235</v>
       </c>
-      <c r="Q38" s="9">
+      <c r="Q38" s="8">
         <f t="shared" si="44"/>
         <v>97.091250000000002</v>
       </c>
-      <c r="R38" s="9">
+      <c r="R38" s="8">
         <f t="shared" si="44"/>
         <v>95.625</v>
       </c>
-      <c r="S38" s="9">
+      <c r="S38" s="8">
         <f t="shared" si="43"/>
         <v>97.282499999999999</v>
       </c>
-      <c r="T38" s="9">
+      <c r="T38" s="8">
         <f t="shared" si="43"/>
         <v>102.31874999999999</v>
       </c>
-      <c r="U38" s="9">
+      <c r="U38" s="8">
         <f t="shared" si="43"/>
         <v>110.73375</v>
       </c>
-      <c r="V38" s="9">
+      <c r="V38" s="8">
         <f t="shared" si="42"/>
         <v>121.57125000000001</v>
       </c>
     </row>
     <row r="39" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B39" s="7">
+      <c r="B39" s="6">
         <v>26</v>
       </c>
       <c r="C39" s="1">
@@ -11245,7 +11245,7 @@
       </c>
     </row>
     <row r="40" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B40" s="7">
+      <c r="B40" s="6">
         <v>27</v>
       </c>
       <c r="C40" s="1">
@@ -11330,7 +11330,7 @@
       </c>
     </row>
     <row r="41" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B41" s="7">
+      <c r="B41" s="6">
         <v>28</v>
       </c>
       <c r="C41" s="1">
@@ -11415,7 +11415,7 @@
       </c>
     </row>
     <row r="42" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B42" s="7">
+      <c r="B42" s="6">
         <v>29</v>
       </c>
       <c r="C42" s="1">
@@ -11500,7 +11500,7 @@
       </c>
     </row>
     <row r="43" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B43" s="7">
+      <c r="B43" s="6">
         <v>30</v>
       </c>
       <c r="C43" s="1">
@@ -11585,7 +11585,7 @@
       </c>
     </row>
     <row r="44" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B44" s="7">
+      <c r="B44" s="6">
         <v>31</v>
       </c>
       <c r="C44" s="1">
@@ -11670,7 +11670,7 @@
       </c>
     </row>
     <row r="45" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B45" s="7">
+      <c r="B45" s="6">
         <v>32</v>
       </c>
       <c r="C45" s="1">
@@ -11755,7 +11755,7 @@
       </c>
     </row>
     <row r="46" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B46" s="7">
+      <c r="B46" s="6">
         <v>33</v>
       </c>
       <c r="C46" s="1">
@@ -11840,7 +11840,7 @@
       </c>
     </row>
     <row r="47" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B47" s="7">
+      <c r="B47" s="6">
         <v>34</v>
       </c>
       <c r="C47" s="1">
@@ -11925,7 +11925,7 @@
       </c>
     </row>
     <row r="48" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B48" s="7">
+      <c r="B48" s="6">
         <v>35</v>
       </c>
       <c r="C48" s="1">
@@ -12010,7 +12010,7 @@
       </c>
     </row>
     <row r="49" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B49" s="7">
+      <c r="B49" s="6">
         <v>36</v>
       </c>
       <c r="C49" s="1">
@@ -12095,7 +12095,7 @@
       </c>
     </row>
     <row r="50" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B50" s="7">
+      <c r="B50" s="6">
         <v>37</v>
       </c>
       <c r="C50" s="1">
@@ -12180,7 +12180,7 @@
       </c>
     </row>
     <row r="51" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B51" s="7">
+      <c r="B51" s="6">
         <v>38</v>
       </c>
       <c r="C51" s="1">
@@ -12265,7 +12265,7 @@
       </c>
     </row>
     <row r="52" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B52" s="7">
+      <c r="B52" s="6">
         <v>39</v>
       </c>
       <c r="C52" s="1">
@@ -12350,7 +12350,7 @@
       </c>
     </row>
     <row r="53" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B53" s="7">
+      <c r="B53" s="6">
         <v>40</v>
       </c>
       <c r="C53" s="1">
@@ -12435,7 +12435,7 @@
       </c>
     </row>
     <row r="54" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B54" s="7">
+      <c r="B54" s="6">
         <v>41</v>
       </c>
       <c r="C54" s="1">
@@ -12520,7 +12520,7 @@
       </c>
     </row>
     <row r="55" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B55" s="7">
+      <c r="B55" s="6">
         <v>42</v>
       </c>
       <c r="C55" s="1">
@@ -12605,7 +12605,7 @@
       </c>
     </row>
     <row r="56" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B56" s="7">
+      <c r="B56" s="6">
         <v>43</v>
       </c>
       <c r="C56" s="1">
@@ -12690,7 +12690,7 @@
       </c>
     </row>
     <row r="57" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B57" s="7">
+      <c r="B57" s="6">
         <v>44</v>
       </c>
       <c r="C57" s="1">
@@ -12775,7 +12775,7 @@
       </c>
     </row>
     <row r="58" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B58" s="7">
+      <c r="B58" s="6">
         <v>45</v>
       </c>
       <c r="C58" s="1">
@@ -12860,7 +12860,7 @@
       </c>
     </row>
     <row r="59" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B59" s="7">
+      <c r="B59" s="6">
         <v>46</v>
       </c>
       <c r="C59" s="1">
@@ -12945,7 +12945,7 @@
       </c>
     </row>
     <row r="60" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B60" s="7">
+      <c r="B60" s="6">
         <v>47</v>
       </c>
       <c r="C60" s="1">
@@ -13030,7 +13030,7 @@
       </c>
     </row>
     <row r="61" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B61" s="7">
+      <c r="B61" s="6">
         <v>48</v>
       </c>
       <c r="C61" s="1">
@@ -13115,7 +13115,7 @@
       </c>
     </row>
     <row r="62" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B62" s="7">
+      <c r="B62" s="6">
         <v>49</v>
       </c>
       <c r="C62" s="1">
@@ -13200,92 +13200,92 @@
       </c>
     </row>
     <row r="63" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B63" s="8">
+      <c r="B63" s="7">
         <v>50</v>
       </c>
-      <c r="C63" s="9">
+      <c r="C63" s="8">
         <f t="shared" si="48"/>
         <v>139.35750000000002</v>
       </c>
-      <c r="D63" s="9">
+      <c r="D63" s="8">
         <f t="shared" si="48"/>
         <v>161.0325</v>
       </c>
-      <c r="E63" s="9">
+      <c r="E63" s="8">
         <f t="shared" si="48"/>
         <v>177.86250000000001</v>
       </c>
-      <c r="F63" s="9">
+      <c r="F63" s="8">
         <f t="shared" si="48"/>
         <v>187.935</v>
       </c>
-      <c r="G63" s="9">
+      <c r="G63" s="8">
         <f t="shared" si="48"/>
         <v>191.25</v>
       </c>
-      <c r="H63" s="9">
+      <c r="H63" s="8">
         <f t="shared" si="48"/>
         <v>188.3175</v>
       </c>
-      <c r="I63" s="9">
+      <c r="I63" s="8">
         <f t="shared" si="48"/>
         <v>180.03</v>
       </c>
-      <c r="J63" s="9">
+      <c r="J63" s="8">
         <f t="shared" si="48"/>
         <v>167.91750000000002</v>
       </c>
-      <c r="K63" s="9">
+      <c r="K63" s="8">
         <f t="shared" si="48"/>
         <v>152.8725</v>
       </c>
-      <c r="L63" s="9">
+      <c r="L63" s="8">
         <f t="shared" si="48"/>
         <v>136.16999999999999</v>
       </c>
-      <c r="M63" s="9">
+      <c r="M63" s="8">
         <f t="shared" si="48"/>
         <v>118.83000000000001</v>
       </c>
-      <c r="N63" s="9">
+      <c r="N63" s="8">
         <f t="shared" si="48"/>
         <v>102.1275</v>
       </c>
-      <c r="O63" s="9">
+      <c r="O63" s="8">
         <f t="shared" si="48"/>
         <v>87.08250000000001</v>
       </c>
-      <c r="P63" s="9">
+      <c r="P63" s="8">
         <f t="shared" si="48"/>
         <v>74.97</v>
       </c>
-      <c r="Q63" s="9">
+      <c r="Q63" s="8">
         <f t="shared" si="48"/>
         <v>66.682500000000005</v>
       </c>
-      <c r="R63" s="9">
+      <c r="R63" s="8">
         <f t="shared" si="48"/>
         <v>63.75</v>
       </c>
-      <c r="S63" s="9">
+      <c r="S63" s="8">
         <f t="shared" si="47"/>
         <v>67.064999999999998</v>
       </c>
-      <c r="T63" s="9">
+      <c r="T63" s="8">
         <f t="shared" si="47"/>
         <v>77.137500000000003</v>
       </c>
-      <c r="U63" s="9">
+      <c r="U63" s="8">
         <f t="shared" si="47"/>
         <v>93.967500000000001</v>
       </c>
-      <c r="V63" s="9">
+      <c r="V63" s="8">
         <f t="shared" si="42"/>
         <v>115.64250000000001</v>
       </c>
     </row>
     <row r="64" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B64" s="7">
+      <c r="B64" s="6">
         <v>51</v>
       </c>
       <c r="C64" s="1">
@@ -13370,7 +13370,7 @@
       </c>
     </row>
     <row r="65" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B65" s="7">
+      <c r="B65" s="6">
         <v>52</v>
       </c>
       <c r="C65" s="1">
@@ -13455,7 +13455,7 @@
       </c>
     </row>
     <row r="66" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B66" s="7">
+      <c r="B66" s="6">
         <v>53</v>
       </c>
       <c r="C66" s="1">
@@ -13540,7 +13540,7 @@
       </c>
     </row>
     <row r="67" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B67" s="7">
+      <c r="B67" s="6">
         <v>54</v>
       </c>
       <c r="C67" s="1">
@@ -13625,7 +13625,7 @@
       </c>
     </row>
     <row r="68" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B68" s="7">
+      <c r="B68" s="6">
         <v>55</v>
       </c>
       <c r="C68" s="1">
@@ -13710,7 +13710,7 @@
       </c>
     </row>
     <row r="69" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B69" s="7">
+      <c r="B69" s="6">
         <v>56</v>
       </c>
       <c r="C69" s="1">
@@ -13795,7 +13795,7 @@
       </c>
     </row>
     <row r="70" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B70" s="7">
+      <c r="B70" s="6">
         <v>57</v>
       </c>
       <c r="C70" s="1">
@@ -13880,7 +13880,7 @@
       </c>
     </row>
     <row r="71" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B71" s="7">
+      <c r="B71" s="6">
         <v>58</v>
       </c>
       <c r="C71" s="1">
@@ -13965,7 +13965,7 @@
       </c>
     </row>
     <row r="72" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B72" s="7">
+      <c r="B72" s="6">
         <v>59</v>
       </c>
       <c r="C72" s="1">
@@ -14050,7 +14050,7 @@
       </c>
     </row>
     <row r="73" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B73" s="7">
+      <c r="B73" s="6">
         <v>60</v>
       </c>
       <c r="C73" s="1">
@@ -14135,7 +14135,7 @@
       </c>
     </row>
     <row r="74" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B74" s="7">
+      <c r="B74" s="6">
         <v>61</v>
       </c>
       <c r="C74" s="1">
@@ -14220,7 +14220,7 @@
       </c>
     </row>
     <row r="75" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B75" s="7">
+      <c r="B75" s="6">
         <v>62</v>
       </c>
       <c r="C75" s="1">
@@ -14305,7 +14305,7 @@
       </c>
     </row>
     <row r="76" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B76" s="7">
+      <c r="B76" s="6">
         <v>63</v>
       </c>
       <c r="C76" s="1">
@@ -14390,7 +14390,7 @@
       </c>
     </row>
     <row r="77" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B77" s="7">
+      <c r="B77" s="6">
         <v>64</v>
       </c>
       <c r="C77" s="1">
@@ -14475,7 +14475,7 @@
       </c>
     </row>
     <row r="78" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B78" s="7">
+      <c r="B78" s="6">
         <v>65</v>
       </c>
       <c r="C78" s="1">
@@ -14560,7 +14560,7 @@
       </c>
     </row>
     <row r="79" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B79" s="7">
+      <c r="B79" s="6">
         <v>66</v>
       </c>
       <c r="C79" s="1">
@@ -14645,7 +14645,7 @@
       </c>
     </row>
     <row r="80" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B80" s="7">
+      <c r="B80" s="6">
         <v>67</v>
       </c>
       <c r="C80" s="1">
@@ -14730,7 +14730,7 @@
       </c>
     </row>
     <row r="81" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B81" s="7">
+      <c r="B81" s="6">
         <v>68</v>
       </c>
       <c r="C81" s="1">
@@ -14815,7 +14815,7 @@
       </c>
     </row>
     <row r="82" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B82" s="7">
+      <c r="B82" s="6">
         <v>69</v>
       </c>
       <c r="C82" s="1">
@@ -14900,7 +14900,7 @@
       </c>
     </row>
     <row r="83" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B83" s="7">
+      <c r="B83" s="6">
         <v>70</v>
       </c>
       <c r="C83" s="1">
@@ -14985,7 +14985,7 @@
       </c>
     </row>
     <row r="84" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B84" s="7">
+      <c r="B84" s="6">
         <v>71</v>
       </c>
       <c r="C84" s="1">
@@ -15070,7 +15070,7 @@
       </c>
     </row>
     <row r="85" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B85" s="7">
+      <c r="B85" s="6">
         <v>72</v>
       </c>
       <c r="C85" s="1">
@@ -15155,7 +15155,7 @@
       </c>
     </row>
     <row r="86" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B86" s="7">
+      <c r="B86" s="6">
         <v>73</v>
       </c>
       <c r="C86" s="1">
@@ -15240,7 +15240,7 @@
       </c>
     </row>
     <row r="87" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B87" s="7">
+      <c r="B87" s="6">
         <v>74</v>
       </c>
       <c r="C87" s="1">
@@ -15325,7 +15325,7 @@
       </c>
     </row>
     <row r="88" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B88" s="7">
+      <c r="B88" s="6">
         <v>75</v>
       </c>
       <c r="C88" s="1">
@@ -15410,7 +15410,7 @@
       </c>
     </row>
     <row r="89" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B89" s="7">
+      <c r="B89" s="6">
         <v>76</v>
       </c>
       <c r="C89" s="1">
@@ -15495,7 +15495,7 @@
       </c>
     </row>
     <row r="90" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B90" s="7">
+      <c r="B90" s="6">
         <v>77</v>
       </c>
       <c r="C90" s="1">
@@ -15580,7 +15580,7 @@
       </c>
     </row>
     <row r="91" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B91" s="7">
+      <c r="B91" s="6">
         <v>78</v>
       </c>
       <c r="C91" s="1">
@@ -15665,7 +15665,7 @@
       </c>
     </row>
     <row r="92" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B92" s="7">
+      <c r="B92" s="6">
         <v>79</v>
       </c>
       <c r="C92" s="1">
@@ -15750,7 +15750,7 @@
       </c>
     </row>
     <row r="93" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B93" s="7">
+      <c r="B93" s="6">
         <v>80</v>
       </c>
       <c r="C93" s="1">
@@ -15835,7 +15835,7 @@
       </c>
     </row>
     <row r="94" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B94" s="7">
+      <c r="B94" s="6">
         <v>81</v>
       </c>
       <c r="C94" s="1">
@@ -15920,7 +15920,7 @@
       </c>
     </row>
     <row r="95" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B95" s="7">
+      <c r="B95" s="6">
         <v>82</v>
       </c>
       <c r="C95" s="1">
@@ -16005,7 +16005,7 @@
       </c>
     </row>
     <row r="96" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B96" s="7">
+      <c r="B96" s="6">
         <v>83</v>
       </c>
       <c r="C96" s="1">
@@ -16090,7 +16090,7 @@
       </c>
     </row>
     <row r="97" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B97" s="7">
+      <c r="B97" s="6">
         <v>84</v>
       </c>
       <c r="C97" s="1">
@@ -16175,7 +16175,7 @@
       </c>
     </row>
     <row r="98" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B98" s="7">
+      <c r="B98" s="6">
         <v>85</v>
       </c>
       <c r="C98" s="1">
@@ -16260,7 +16260,7 @@
       </c>
     </row>
     <row r="99" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B99" s="7">
+      <c r="B99" s="6">
         <v>86</v>
       </c>
       <c r="C99" s="1">
@@ -16345,7 +16345,7 @@
       </c>
     </row>
     <row r="100" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B100" s="7">
+      <c r="B100" s="6">
         <v>87</v>
       </c>
       <c r="C100" s="1">
@@ -16430,7 +16430,7 @@
       </c>
     </row>
     <row r="101" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B101" s="7">
+      <c r="B101" s="6">
         <v>88</v>
       </c>
       <c r="C101" s="1">
@@ -16515,7 +16515,7 @@
       </c>
     </row>
     <row r="102" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B102" s="7">
+      <c r="B102" s="6">
         <v>89</v>
       </c>
       <c r="C102" s="1">
@@ -16600,7 +16600,7 @@
       </c>
     </row>
     <row r="103" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B103" s="7">
+      <c r="B103" s="6">
         <v>90</v>
       </c>
       <c r="C103" s="1">
@@ -16685,7 +16685,7 @@
       </c>
     </row>
     <row r="104" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B104" s="7">
+      <c r="B104" s="6">
         <v>91</v>
       </c>
       <c r="C104" s="1">
@@ -16770,7 +16770,7 @@
       </c>
     </row>
     <row r="105" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B105" s="7">
+      <c r="B105" s="6">
         <v>92</v>
       </c>
       <c r="C105" s="1">
@@ -16855,7 +16855,7 @@
       </c>
     </row>
     <row r="106" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B106" s="7">
+      <c r="B106" s="6">
         <v>93</v>
       </c>
       <c r="C106" s="1">
@@ -16940,7 +16940,7 @@
       </c>
     </row>
     <row r="107" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B107" s="7">
+      <c r="B107" s="6">
         <v>94</v>
       </c>
       <c r="C107" s="1">
@@ -17025,7 +17025,7 @@
       </c>
     </row>
     <row r="108" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B108" s="7">
+      <c r="B108" s="6">
         <v>95</v>
       </c>
       <c r="C108" s="1">
@@ -17110,7 +17110,7 @@
       </c>
     </row>
     <row r="109" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B109" s="7">
+      <c r="B109" s="6">
         <v>96</v>
       </c>
       <c r="C109" s="1">
@@ -17195,7 +17195,7 @@
       </c>
     </row>
     <row r="110" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B110" s="7">
+      <c r="B110" s="6">
         <v>97</v>
       </c>
       <c r="C110" s="1">
@@ -17280,7 +17280,7 @@
       </c>
     </row>
     <row r="111" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B111" s="7">
+      <c r="B111" s="6">
         <v>98</v>
       </c>
       <c r="C111" s="1">
@@ -17365,7 +17365,7 @@
       </c>
     </row>
     <row r="112" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B112" s="7">
+      <c r="B112" s="6">
         <v>99</v>
       </c>
       <c r="C112" s="1">
@@ -17450,86 +17450,86 @@
       </c>
     </row>
     <row r="113" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B113" s="8">
+      <c r="B113" s="7">
         <v>100</v>
       </c>
-      <c r="C113" s="9">
+      <c r="C113" s="8">
         <f>127.5+(C$11-127.5)*$B113/100</f>
         <v>151.215</v>
       </c>
-      <c r="D113" s="9">
+      <c r="D113" s="8">
         <f t="shared" ref="D113:U113" si="55">127.5+(D$11-127.5)*$B113/100</f>
         <v>194.565</v>
       </c>
-      <c r="E113" s="9">
+      <c r="E113" s="8">
         <f t="shared" si="55"/>
         <v>228.22499999999999</v>
       </c>
-      <c r="F113" s="9">
+      <c r="F113" s="8">
         <f t="shared" si="55"/>
         <v>248.37000000000003</v>
       </c>
-      <c r="G113" s="9">
+      <c r="G113" s="8">
         <f t="shared" si="55"/>
         <v>255</v>
       </c>
-      <c r="H113" s="9">
+      <c r="H113" s="8">
         <f t="shared" si="55"/>
         <v>249.13499999999999</v>
       </c>
-      <c r="I113" s="9">
+      <c r="I113" s="8">
         <f t="shared" si="55"/>
         <v>232.56</v>
       </c>
-      <c r="J113" s="9">
+      <c r="J113" s="8">
         <f t="shared" si="55"/>
         <v>208.33500000000001</v>
       </c>
-      <c r="K113" s="9">
+      <c r="K113" s="8">
         <f t="shared" si="55"/>
         <v>178.245</v>
       </c>
-      <c r="L113" s="9">
+      <c r="L113" s="8">
         <f t="shared" si="55"/>
         <v>144.83999999999997</v>
       </c>
-      <c r="M113" s="9">
+      <c r="M113" s="8">
         <f t="shared" si="55"/>
         <v>110.16000000000001</v>
       </c>
-      <c r="N113" s="9">
+      <c r="N113" s="8">
         <f t="shared" si="55"/>
         <v>76.754999999999995</v>
       </c>
-      <c r="O113" s="9">
+      <c r="O113" s="8">
         <f t="shared" si="55"/>
         <v>46.665000000000006</v>
       </c>
-      <c r="P113" s="9">
+      <c r="P113" s="8">
         <f t="shared" si="55"/>
         <v>22.439999999999998</v>
       </c>
-      <c r="Q113" s="9">
+      <c r="Q113" s="8">
         <f t="shared" si="55"/>
         <v>5.8649999999999949</v>
       </c>
-      <c r="R113" s="9">
+      <c r="R113" s="8">
         <f t="shared" si="55"/>
         <v>0</v>
       </c>
-      <c r="S113" s="9">
+      <c r="S113" s="8">
         <f t="shared" si="55"/>
         <v>6.6299999999999955</v>
       </c>
-      <c r="T113" s="9">
+      <c r="T113" s="8">
         <f t="shared" si="55"/>
         <v>26.775000000000006</v>
       </c>
-      <c r="U113" s="9">
+      <c r="U113" s="8">
         <f t="shared" si="55"/>
         <v>60.435000000000002</v>
       </c>
-      <c r="V113" s="9">
+      <c r="V113" s="8">
         <f>127.5+(V$11-127.5)*$B113/100</f>
         <v>103.78500000000001</v>
       </c>

</xml_diff>